<commit_message>
📊 Update confusion matrices & add dual examples for detection/classification
Changes:
- Updated confusion matrix section to show 8 matrices (top 2 models per dataset)
- Expanded narrative with detailed per-dataset analysis (5 paragraphs)
- Added 2nd detection example: MD-2019 Stages (6 parasites, 81.6% conf)
- Added 2nd classification example: MD-2019 Stages (5 parasites, 100% acc)
- Updated captions: Gambar 1a-b (detection), Gambar 6a-b (classification)

Top 2 models per dataset (by balanced accuracy):
- IML Lifecycle: DenseNet121 (93.79%), EfficientNet-B2 (91.96%)
- MP-IDB Species: ResNet101 (88.10%), EfficientNet-B1 (86.43%)
- MP-IDB Stages: ResNet101 (76.99%), EfficientNet-B0 (73.78%)
- MD-2019 Stages: EfficientNet-B0 (85.51%), EfficientNet-B1 (83.91%)

Files modified:
- luaran/laporan_akhir/Laporan_Akhir_Penelitian.md
- visualization_outputs/report_examples/ (2 new images)

Generated with Claude Code
</commit_message>
<xml_diff>
--- a/luaran/laporan_akhir/tables/Table1_Dataset_Statistics.xlsx
+++ b/luaran/laporan_akhir/tables/Table1_Dataset_Statistics.xlsx
@@ -94,7 +94,7 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -103,7 +103,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -532,7 +532,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>iml_lifecycle</t>
+          <t>IML Lifecycle</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
@@ -564,7 +564,7 @@
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>md_2019_stages</t>
+          <t>MD-2019 Stages</t>
         </is>
       </c>
       <c r="B3" s="6" t="n">
@@ -596,7 +596,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>mp_idb_species</t>
+          <t>MP-IDB Species</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
@@ -628,7 +628,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>mp_idb_stages</t>
+          <t>MP-IDB Stages</t>
         </is>
       </c>
       <c r="B5" s="6" t="n">

</xml_diff>